<commit_message>
Bugfix + Final calcs
Fixed some more bugs that were reported in the github and this is also the version that has the final calcs for Pearl alongside the teams used for all of these calcs.
</commit_message>
<xml_diff>
--- a/TeamCalcs_SheetExport.xlsx
+++ b/TeamCalcs_SheetExport.xlsx
@@ -456,84 +456,84 @@
     <row r="9">
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>112184.255</t>
+          <t>76786.492</t>
         </is>
       </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
-          <t>105101.699</t>
+          <t>70413.337</t>
         </is>
       </c>
       <c r="K9" s="1" t="inlineStr">
         <is>
-          <t>117962.780</t>
+          <t>83474.925</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>error margin: +/-0.48%</t>
+          <t>error margin: +/-0.74%</t>
         </is>
       </c>
       <c r="R9" s="1" t="inlineStr">
         <is>
-          <t>124927.721</t>
+          <t>83555.088</t>
         </is>
       </c>
       <c r="T9" s="1" t="inlineStr">
         <is>
-          <t>115745.095</t>
+          <t>79196.481</t>
         </is>
       </c>
       <c r="V9" s="1" t="inlineStr">
         <is>
-          <t>130262.723</t>
+          <t>87216.702</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>error margin: +/-0.50%</t>
+          <t>error margin: +/-0.43%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 30726958.215  (64.0% of Evanescia's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 17468895.875  (59.8% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 3245783.425  (66.5% of ElationMC's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 3349822.915  (64.0% of ElationMC's DMG)</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 6078500.295  (73.4% of YaoGuang's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 5743271.415  (75.7% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 107184.545  (64.1% of Pearl's DMG)</t>
+          <t>- ELABANGER  avg DMG: 68301.665  (57.5% of Pearl's DMG)</t>
         </is>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 34751457.909  (64.6% of Evanescia's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 18728986.878  (58.7% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 3501443.185  (66.6% of ElationMC's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 3624443.779  (64.1% of ElationMC's DMG)</t>
         </is>
       </c>
       <c r="V12" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 6558126.195  (72.4% of YaoGuang's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 6198123.241  (75.7% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 122841.786  (56.6% of Pearl's DMG)</t>
+          <t>- BSC  avg DMG: 80566.455  (50.2% of Pearl's DMG)</t>
         </is>
       </c>
     </row>
@@ -541,42 +541,42 @@
     <row r="14">
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 13777758.862  (28.7% of Evanescia's DMG)</t>
+          <t>- ELABANGER  avg DMG: 10701882.514  (36.6% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 1517309.852  (31.1% of ElationMC's DMG)</t>
+          <t>- ELABANGER  avg DMG: 1773795.778  (33.9% of ElationMC's DMG)</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 2101946.974  (25.4% of YaoGuang's DMG)</t>
+          <t>- ELABANGER  avg DMG: 1819001.637  (24.0% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>- BSC  avg DMG: 60052.310  (35.9% of Pearl's DMG)</t>
+          <t>- BSC  avg DMG: 50435.214  (42.5% of Pearl's DMG)</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 14817706.028  (27.5% of Evanescia's DMG)</t>
+          <t>- ELABANGER  avg DMG: 11874300.871  (37.2% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 1620133.121  (30.8% of ElationMC's DMG)</t>
+          <t>- ELABANGER  avg DMG: 1895713.976  (33.5% of ElationMC's DMG)</t>
         </is>
       </c>
       <c r="V14" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 2368527.607  (26.2% of YaoGuang's DMG)</t>
+          <t>- ELABANGER  avg DMG: 1955394.644  (23.9% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>- BSC  avg DMG: 94257.009  (43.4% of Pearl's DMG)</t>
+          <t>- ELABANGER  avg DMG: 80074.767  (49.8% of Pearl's DMG)</t>
         </is>
       </c>
     </row>
@@ -584,17 +584,17 @@
     <row r="16">
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>- ULT  avg DMG: 1908102.496  (4.0% of Evanescia's DMG)</t>
+          <t>- BSC  avg DMG: 598775.127  (2.0% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>- SKL  avg DMG: 117271.892  (2.4% of ElationMC's DMG)</t>
+          <t>- SKL  avg DMG: 111690.232  (2.1% of ElationMC's DMG)</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>- BRK  avg DMG: 66965.746  (0.8% of YaoGuang's DMG)</t>
+          <t>- BSC  avg DMG: 26505.789  (0.3% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -604,17 +604,17 @@
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>- ULT  avg DMG: 2305622.703  (4.3% of Evanescia's DMG)</t>
+          <t>- BSC  avg DMG: 732907.267  (2.3% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>- SKL  avg DMG: 133642.308  (2.5% of ElationMC's DMG)</t>
+          <t>- SKL  avg DMG: 130362.433  (2.3% of ElationMC's DMG)</t>
         </is>
       </c>
       <c r="V16" s="3" t="inlineStr">
         <is>
-          <t>- BRK  avg DMG: 89162.625  (1.0% of YaoGuang's DMG)</t>
+          <t>- BSC  avg DMG: 30558.393  (0.4% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="X16" s="3" t="inlineStr">
@@ -627,54 +627,54 @@
     <row r="18">
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>Evanescia</t>
+          <t>Sparxie</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>87330.399</t>
+          <t>53149.838</t>
         </is>
       </c>
       <c r="X18" s="4" t="inlineStr">
         <is>
-          <t>Evanescia</t>
+          <t>Sparxie</t>
         </is>
       </c>
       <c r="Y18" s="4" t="inlineStr">
         <is>
-          <t>97823.474</t>
+          <t>57986.129</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>4328429.3</t>
+          <t>8675940.8</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>760333.5</t>
+          <t>6792929.7</t>
         </is>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>2036510.8</t>
+          <t>306704.0</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>28012.0</t>
+          <t>5881.5</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
         <is>
-          <t>754173.2</t>
+          <t>1279383.4</t>
         </is>
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
-          <t>749399.8</t>
+          <t>291042.2</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
@@ -684,37 +684,37 @@
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>8873.391</t>
+          <t>9518.744</t>
         </is>
       </c>
       <c r="R19" s="1" t="inlineStr">
         <is>
-          <t>4773518.3</t>
+          <t>10276560.2</t>
         </is>
       </c>
       <c r="S19" s="1" t="inlineStr">
         <is>
-          <t>805119.3</t>
+          <t>8248884.1</t>
         </is>
       </c>
       <c r="T19" s="1" t="inlineStr">
         <is>
-          <t>2100906.3</t>
+          <t>287312.9</t>
         </is>
       </c>
       <c r="U19" s="1" t="inlineStr">
         <is>
-          <t>82697.7</t>
+          <t>22062.2</t>
         </is>
       </c>
       <c r="V19" s="1" t="inlineStr">
         <is>
-          <t>891957.3</t>
+          <t>1287393.3</t>
         </is>
       </c>
       <c r="W19" s="1" t="inlineStr">
         <is>
-          <t>892837.8</t>
+          <t>430907.7</t>
         </is>
       </c>
       <c r="X19" s="4" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="Y19" s="4" t="inlineStr">
         <is>
-          <t>9554.943</t>
+          <t>10273.673</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>15054.120</t>
+          <t>13797.780</t>
         </is>
       </c>
       <c r="X20" s="4" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="Y20" s="4" t="inlineStr">
         <is>
-          <t>16459.682</t>
+          <t>14880.139</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>304.067</t>
+          <t>215.885</t>
         </is>
       </c>
       <c r="X21" s="4" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="Y21" s="4" t="inlineStr">
         <is>
-          <t>394.725</t>
+          <t>292.075</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug fixes + Aventurine Waveflair
Fixed some more bugs mostly related to elation such as in Yao Guang kit mostly and a bit in ElationMC and Pearl. Also started work on Aventurine Waveflair. Should be done relatively soon and then gonna work on Aha.
</commit_message>
<xml_diff>
--- a/TeamCalcs_SheetExport.xlsx
+++ b/TeamCalcs_SheetExport.xlsx
@@ -450,90 +450,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="G9:Y21"/>
+  <dimension ref="G9:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="9">
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>76786.492</t>
+          <t>86613.032</t>
         </is>
       </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
-          <t>70413.337</t>
+          <t>76420.889</t>
         </is>
       </c>
       <c r="K9" s="1" t="inlineStr">
         <is>
-          <t>83474.925</t>
+          <t>100127.491</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>error margin: +/-0.74%</t>
-        </is>
-      </c>
-      <c r="R9" s="1" t="inlineStr">
-        <is>
-          <t>83555.088</t>
-        </is>
-      </c>
-      <c r="T9" s="1" t="inlineStr">
-        <is>
-          <t>79196.481</t>
-        </is>
-      </c>
-      <c r="V9" s="1" t="inlineStr">
-        <is>
-          <t>87216.702</t>
-        </is>
-      </c>
-      <c r="X9" s="2" t="inlineStr">
-        <is>
-          <t>error margin: +/-0.43%</t>
+          <t>error margin: +/-1.07%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 17468895.875  (59.8% of Sparxie's DMG)</t>
+          <t>- ELABANGER  avg DMG: 29390484.863  (86.5% of SilverWolf999's DMG)</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 3349822.915  (64.0% of ElationMC's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 5601962.174  (63.2% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>- ELAPUNCH  avg DMG: 5743271.415  (75.7% of YaoGuang's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 3359353.570  (71.2% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 68301.665  (57.5% of Pearl's DMG)</t>
-        </is>
-      </c>
-      <c r="R12" s="3" t="inlineStr">
-        <is>
-          <t>- ELAPUNCH  avg DMG: 18728986.878  (58.7% of Sparxie's DMG)</t>
-        </is>
-      </c>
-      <c r="T12" s="3" t="inlineStr">
-        <is>
-          <t>- ELAPUNCH  avg DMG: 3624443.779  (64.1% of ElationMC's DMG)</t>
-        </is>
-      </c>
-      <c r="V12" s="3" t="inlineStr">
-        <is>
-          <t>- ELAPUNCH  avg DMG: 6198123.241  (75.7% of YaoGuang's DMG)</t>
-        </is>
-      </c>
-      <c r="X12" s="3" t="inlineStr">
-        <is>
-          <t>- BSC  avg DMG: 80566.455  (50.2% of Pearl's DMG)</t>
+          <t>- ELABANGER  avg DMG: 48980.375  (61.5% of Pearl's DMG)</t>
         </is>
       </c>
     </row>
@@ -541,42 +501,22 @@
     <row r="14">
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 10701882.514  (36.6% of Sparxie's DMG)</t>
+          <t>- ELAPUNCH  avg DMG: 4448586.842  (13.1% of SilverWolf999's DMG)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 1773795.778  (33.9% of ElationMC's DMG)</t>
+          <t>- ELABANGER  avg DMG: 2953835.107  (33.3% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>- ELABANGER  avg DMG: 1819001.637  (24.0% of YaoGuang's DMG)</t>
+          <t>- ELABANGER  avg DMG: 1329900.849  (28.2% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>- BSC  avg DMG: 50435.214  (42.5% of Pearl's DMG)</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>- ELABANGER  avg DMG: 11874300.871  (37.2% of Sparxie's DMG)</t>
-        </is>
-      </c>
-      <c r="T14" s="3" t="inlineStr">
-        <is>
-          <t>- ELABANGER  avg DMG: 1895713.976  (33.5% of ElationMC's DMG)</t>
-        </is>
-      </c>
-      <c r="V14" s="3" t="inlineStr">
-        <is>
-          <t>- ELABANGER  avg DMG: 1955394.644  (23.9% of YaoGuang's DMG)</t>
-        </is>
-      </c>
-      <c r="X14" s="3" t="inlineStr">
-        <is>
-          <t>- ELABANGER  avg DMG: 80074.767  (49.8% of Pearl's DMG)</t>
+          <t>- BSC  avg DMG: 30663.013  (38.5% of Pearl's DMG)</t>
         </is>
       </c>
     </row>
@@ -584,40 +524,20 @@
     <row r="16">
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>- BSC  avg DMG: 598775.127  (2.0% of Sparxie's DMG)</t>
+          <t>- SKL  avg DMG: 93999.533  (0.3% of SilverWolf999's DMG)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>- SKL  avg DMG: 111690.232  (2.1% of ElationMC's DMG)</t>
+          <t>- BSC  avg DMG: 250361.503  (2.8% of Sparxie's DMG)</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>- BSC  avg DMG: 26505.789  (0.3% of YaoGuang's DMG)</t>
+          <t>- BSC  avg DMG: 26310.959  (0.6% of YaoGuang's DMG)</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
-        <is>
-          <t>- SKL  avg DMG: 0.000  (0.0% of Pearl's DMG)</t>
-        </is>
-      </c>
-      <c r="R16" s="3" t="inlineStr">
-        <is>
-          <t>- BSC  avg DMG: 732907.267  (2.3% of Sparxie's DMG)</t>
-        </is>
-      </c>
-      <c r="T16" s="3" t="inlineStr">
-        <is>
-          <t>- SKL  avg DMG: 130362.433  (2.3% of ElationMC's DMG)</t>
-        </is>
-      </c>
-      <c r="V16" s="3" t="inlineStr">
-        <is>
-          <t>- BSC  avg DMG: 30558.393  (0.4% of YaoGuang's DMG)</t>
-        </is>
-      </c>
-      <c r="X16" s="3" t="inlineStr">
         <is>
           <t>- SKL  avg DMG: 0.000  (0.0% of Pearl's DMG)</t>
         </is>
@@ -627,104 +547,54 @@
     <row r="18">
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>Sparxie</t>
+          <t>SilverWolf999</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>53149.838</t>
-        </is>
-      </c>
-      <c r="X18" s="4" t="inlineStr">
-        <is>
-          <t>Sparxie</t>
-        </is>
-      </c>
-      <c r="Y18" s="4" t="inlineStr">
-        <is>
-          <t>57986.129</t>
+          <t>61786.112</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>8675940.8</t>
+          <t>847561.8</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>6792929.7</t>
+          <t>556397.3</t>
         </is>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>306704.0</t>
+          <t>93554.9</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>5881.5</t>
+          <t>197609.7</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
         <is>
-          <t>1279383.4</t>
+          <t>/</t>
         </is>
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
-          <t>291042.2</t>
+          <t>/</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>ElationMC</t>
+          <t>Sparxie</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>9518.744</t>
-        </is>
-      </c>
-      <c r="R19" s="1" t="inlineStr">
-        <is>
-          <t>10276560.2</t>
-        </is>
-      </c>
-      <c r="S19" s="1" t="inlineStr">
-        <is>
-          <t>8248884.1</t>
-        </is>
-      </c>
-      <c r="T19" s="1" t="inlineStr">
-        <is>
-          <t>287312.9</t>
-        </is>
-      </c>
-      <c r="U19" s="1" t="inlineStr">
-        <is>
-          <t>22062.2</t>
-        </is>
-      </c>
-      <c r="V19" s="1" t="inlineStr">
-        <is>
-          <t>1287393.3</t>
-        </is>
-      </c>
-      <c r="W19" s="1" t="inlineStr">
-        <is>
-          <t>430907.7</t>
-        </is>
-      </c>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>ElationMC</t>
-        </is>
-      </c>
-      <c r="Y19" s="4" t="inlineStr">
-        <is>
-          <t>10273.673</t>
+          <t>16108.359</t>
         </is>
       </c>
     </row>
@@ -736,17 +606,7 @@
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>13797.780</t>
-        </is>
-      </c>
-      <c r="X20" s="4" t="inlineStr">
-        <is>
-          <t>YaoGuang</t>
-        </is>
-      </c>
-      <c r="Y20" s="4" t="inlineStr">
-        <is>
-          <t>14880.139</t>
+          <t>8573.755</t>
         </is>
       </c>
     </row>
@@ -758,63 +618,31 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>215.885</t>
-        </is>
-      </c>
-      <c r="X21" s="4" t="inlineStr">
-        <is>
-          <t>Pearl</t>
-        </is>
-      </c>
-      <c r="Y21" s="4" t="inlineStr">
-        <is>
-          <t>292.075</t>
+          <t>144.806</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="44">
-    <mergeCell ref="R19:R20"/>
+  <mergeCells count="22">
     <mergeCell ref="M16:N17"/>
-    <mergeCell ref="R12:S13"/>
-    <mergeCell ref="T12:U13"/>
     <mergeCell ref="I12:J13"/>
     <mergeCell ref="K12:L13"/>
     <mergeCell ref="M12:N13"/>
     <mergeCell ref="K9:L9"/>
     <mergeCell ref="M9:N9"/>
-    <mergeCell ref="V19:V20"/>
     <mergeCell ref="G14:H15"/>
     <mergeCell ref="G19:G20"/>
     <mergeCell ref="I14:J15"/>
     <mergeCell ref="K14:L15"/>
     <mergeCell ref="M14:N15"/>
-    <mergeCell ref="S19:S20"/>
-    <mergeCell ref="X14:Y15"/>
     <mergeCell ref="J19:J20"/>
-    <mergeCell ref="V16:W17"/>
-    <mergeCell ref="V12:W13"/>
     <mergeCell ref="G16:H17"/>
-    <mergeCell ref="T9:U9"/>
-    <mergeCell ref="T16:U17"/>
-    <mergeCell ref="V9:W9"/>
-    <mergeCell ref="R14:S15"/>
     <mergeCell ref="H19:H20"/>
-    <mergeCell ref="X9:Y9"/>
     <mergeCell ref="K16:L17"/>
     <mergeCell ref="G12:H13"/>
-    <mergeCell ref="X12:Y13"/>
-    <mergeCell ref="V14:W15"/>
     <mergeCell ref="I19:I20"/>
-    <mergeCell ref="T19:T20"/>
     <mergeCell ref="K19:K20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="T14:U15"/>
-    <mergeCell ref="R16:S17"/>
-    <mergeCell ref="X16:Y17"/>
     <mergeCell ref="I16:J17"/>
-    <mergeCell ref="R9:S9"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="L19:L20"/>

</xml_diff>